<commit_message>
added the inside interpolation
</commit_message>
<xml_diff>
--- a/data/merged_panel_long.xlsx
+++ b/data/merged_panel_long.xlsx
@@ -5109,9 +5109,7 @@
       <c r="E142" t="n">
         <v>1990</v>
       </c>
-      <c r="F142" t="n">
-        <v>10.272</v>
-      </c>
+      <c r="F142" t="inlineStr"/>
       <c r="G142" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -7419,9 +7417,7 @@
       <c r="E212" t="n">
         <v>1990</v>
       </c>
-      <c r="F212" t="n">
-        <v>-11.69999848202703</v>
-      </c>
+      <c r="F212" t="inlineStr"/>
       <c r="G212" t="inlineStr">
         <is>
           <t>GDP Growth Rate</t>
@@ -9729,9 +9725,7 @@
       <c r="E282" t="n">
         <v>1990</v>
       </c>
-      <c r="F282" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F282" t="inlineStr"/>
       <c r="G282" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9762,9 +9756,7 @@
       <c r="E283" t="n">
         <v>1991</v>
       </c>
-      <c r="F283" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F283" t="inlineStr"/>
       <c r="G283" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9795,9 +9787,7 @@
       <c r="E284" t="n">
         <v>1992</v>
       </c>
-      <c r="F284" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F284" t="inlineStr"/>
       <c r="G284" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9828,9 +9818,7 @@
       <c r="E285" t="n">
         <v>1993</v>
       </c>
-      <c r="F285" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F285" t="inlineStr"/>
       <c r="G285" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9861,9 +9849,7 @@
       <c r="E286" t="n">
         <v>1994</v>
       </c>
-      <c r="F286" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F286" t="inlineStr"/>
       <c r="G286" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9894,9 +9880,7 @@
       <c r="E287" t="n">
         <v>1995</v>
       </c>
-      <c r="F287" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F287" t="inlineStr"/>
       <c r="G287" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9927,9 +9911,7 @@
       <c r="E288" t="n">
         <v>1996</v>
       </c>
-      <c r="F288" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F288" t="inlineStr"/>
       <c r="G288" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9960,9 +9942,7 @@
       <c r="E289" t="n">
         <v>1997</v>
       </c>
-      <c r="F289" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F289" t="inlineStr"/>
       <c r="G289" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -9993,9 +9973,7 @@
       <c r="E290" t="n">
         <v>1998</v>
       </c>
-      <c r="F290" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F290" t="inlineStr"/>
       <c r="G290" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -10026,9 +10004,7 @@
       <c r="E291" t="n">
         <v>1999</v>
       </c>
-      <c r="F291" t="n">
-        <v>36.458179473877</v>
-      </c>
+      <c r="F291" t="inlineStr"/>
       <c r="G291" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -12039,9 +12015,7 @@
       <c r="E352" t="n">
         <v>1990</v>
       </c>
-      <c r="F352" t="n">
-        <v>2.351</v>
-      </c>
+      <c r="F352" t="inlineStr"/>
       <c r="G352" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -16659,9 +16633,7 @@
       <c r="E492" t="n">
         <v>1990</v>
       </c>
-      <c r="F492" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F492" t="inlineStr"/>
       <c r="G492" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16692,9 +16664,7 @@
       <c r="E493" t="n">
         <v>1991</v>
       </c>
-      <c r="F493" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F493" t="inlineStr"/>
       <c r="G493" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16725,9 +16695,7 @@
       <c r="E494" t="n">
         <v>1992</v>
       </c>
-      <c r="F494" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F494" t="inlineStr"/>
       <c r="G494" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16758,9 +16726,7 @@
       <c r="E495" t="n">
         <v>1993</v>
       </c>
-      <c r="F495" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F495" t="inlineStr"/>
       <c r="G495" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16791,9 +16757,7 @@
       <c r="E496" t="n">
         <v>1994</v>
       </c>
-      <c r="F496" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F496" t="inlineStr"/>
       <c r="G496" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16824,9 +16788,7 @@
       <c r="E497" t="n">
         <v>1995</v>
       </c>
-      <c r="F497" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F497" t="inlineStr"/>
       <c r="G497" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16857,9 +16819,7 @@
       <c r="E498" t="n">
         <v>1996</v>
       </c>
-      <c r="F498" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F498" t="inlineStr"/>
       <c r="G498" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16890,9 +16850,7 @@
       <c r="E499" t="n">
         <v>1997</v>
       </c>
-      <c r="F499" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F499" t="inlineStr"/>
       <c r="G499" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16923,9 +16881,7 @@
       <c r="E500" t="n">
         <v>1998</v>
       </c>
-      <c r="F500" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F500" t="inlineStr"/>
       <c r="G500" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16956,9 +16912,7 @@
       <c r="E501" t="n">
         <v>1999</v>
       </c>
-      <c r="F501" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F501" t="inlineStr"/>
       <c r="G501" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -16989,9 +16943,7 @@
       <c r="E502" t="n">
         <v>2000</v>
       </c>
-      <c r="F502" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F502" t="inlineStr"/>
       <c r="G502" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -17022,9 +16974,7 @@
       <c r="E503" t="n">
         <v>2001</v>
       </c>
-      <c r="F503" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F503" t="inlineStr"/>
       <c r="G503" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -17055,9 +17005,7 @@
       <c r="E504" t="n">
         <v>2002</v>
       </c>
-      <c r="F504" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F504" t="inlineStr"/>
       <c r="G504" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -17088,9 +17036,7 @@
       <c r="E505" t="n">
         <v>2003</v>
       </c>
-      <c r="F505" t="n">
-        <v>19.9779891967773</v>
-      </c>
+      <c r="F505" t="inlineStr"/>
       <c r="G505" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -18969,9 +18915,7 @@
       <c r="E562" t="n">
         <v>1990</v>
       </c>
-      <c r="F562" t="n">
-        <v>16.577</v>
-      </c>
+      <c r="F562" t="inlineStr"/>
       <c r="G562" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -25899,9 +25843,7 @@
       <c r="E772" t="n">
         <v>1990</v>
       </c>
-      <c r="F772" t="n">
-        <v>21.089</v>
-      </c>
+      <c r="F772" t="inlineStr"/>
       <c r="G772" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -30519,9 +30461,7 @@
       <c r="E912" t="n">
         <v>1990</v>
       </c>
-      <c r="F912" t="n">
-        <v>34.0329704284668</v>
-      </c>
+      <c r="F912" t="inlineStr"/>
       <c r="G912" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -31641,9 +31581,7 @@
       <c r="E946" t="n">
         <v>2024</v>
       </c>
-      <c r="F946" t="n">
-        <v>84.09585629400109</v>
-      </c>
+      <c r="F946" t="inlineStr"/>
       <c r="G946" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -32829,9 +32767,7 @@
       <c r="E982" t="n">
         <v>1990</v>
       </c>
-      <c r="F982" t="n">
-        <v>2.558</v>
-      </c>
+      <c r="F982" t="inlineStr"/>
       <c r="G982" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -37449,9 +37385,7 @@
       <c r="E1122" t="n">
         <v>1990</v>
       </c>
-      <c r="F1122" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1122" t="inlineStr"/>
       <c r="G1122" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -37482,9 +37416,7 @@
       <c r="E1123" t="n">
         <v>1991</v>
       </c>
-      <c r="F1123" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1123" t="inlineStr"/>
       <c r="G1123" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -37515,9 +37447,7 @@
       <c r="E1124" t="n">
         <v>1992</v>
       </c>
-      <c r="F1124" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1124" t="inlineStr"/>
       <c r="G1124" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -37548,9 +37478,7 @@
       <c r="E1125" t="n">
         <v>1993</v>
       </c>
-      <c r="F1125" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1125" t="inlineStr"/>
       <c r="G1125" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -37581,9 +37509,7 @@
       <c r="E1126" t="n">
         <v>1994</v>
       </c>
-      <c r="F1126" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1126" t="inlineStr"/>
       <c r="G1126" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -37614,9 +37540,7 @@
       <c r="E1127" t="n">
         <v>1995</v>
       </c>
-      <c r="F1127" t="n">
-        <v>14.3763198852539</v>
-      </c>
+      <c r="F1127" t="inlineStr"/>
       <c r="G1127" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -38538,9 +38462,7 @@
       <c r="E1155" t="n">
         <v>2023</v>
       </c>
-      <c r="F1155" t="n">
-        <v>59.131290435791</v>
-      </c>
+      <c r="F1155" t="inlineStr"/>
       <c r="G1155" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -38571,9 +38493,7 @@
       <c r="E1156" t="n">
         <v>2024</v>
       </c>
-      <c r="F1156" t="n">
-        <v>59.131290435791</v>
-      </c>
+      <c r="F1156" t="inlineStr"/>
       <c r="G1156" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -39759,9 +39679,7 @@
       <c r="E1192" t="n">
         <v>1990</v>
       </c>
-      <c r="F1192" t="n">
-        <v>24.598</v>
-      </c>
+      <c r="F1192" t="inlineStr"/>
       <c r="G1192" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -46689,9 +46607,7 @@
       <c r="E1402" t="n">
         <v>1990</v>
       </c>
-      <c r="F1402" t="n">
-        <v>32.183</v>
-      </c>
+      <c r="F1402" t="inlineStr"/>
       <c r="G1402" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -50121,9 +50037,7 @@
       <c r="E1506" t="n">
         <v>2024</v>
       </c>
-      <c r="F1506" t="n">
-        <v>-0.7605844702573137</v>
-      </c>
+      <c r="F1506" t="inlineStr"/>
       <c r="G1506" t="inlineStr">
         <is>
           <t>GDP Growth Rate</t>
@@ -51276,9 +51190,7 @@
       <c r="E1541" t="n">
         <v>2024</v>
       </c>
-      <c r="F1541" t="n">
-        <v>3477.724898426838</v>
-      </c>
+      <c r="F1541" t="inlineStr"/>
       <c r="G1541" t="inlineStr">
         <is>
           <t>GDP per Capita</t>
@@ -51309,9 +51221,7 @@
       <c r="E1542" t="n">
         <v>1990</v>
       </c>
-      <c r="F1542" t="n">
-        <v>23.0771808624268</v>
-      </c>
+      <c r="F1542" t="inlineStr"/>
       <c r="G1542" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -51342,9 +51252,7 @@
       <c r="E1543" t="n">
         <v>1991</v>
       </c>
-      <c r="F1543" t="n">
-        <v>23.0771808624268</v>
-      </c>
+      <c r="F1543" t="inlineStr"/>
       <c r="G1543" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -52299,9 +52207,7 @@
       <c r="E1572" t="n">
         <v>2020</v>
       </c>
-      <c r="F1572" t="n">
-        <v>57.1435211987779</v>
-      </c>
+      <c r="F1572" t="inlineStr"/>
       <c r="G1572" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -52332,9 +52238,7 @@
       <c r="E1573" t="n">
         <v>2021</v>
       </c>
-      <c r="F1573" t="n">
-        <v>57.1435211987779</v>
-      </c>
+      <c r="F1573" t="inlineStr"/>
       <c r="G1573" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -52365,9 +52269,7 @@
       <c r="E1574" t="n">
         <v>2022</v>
       </c>
-      <c r="F1574" t="n">
-        <v>57.1435211987779</v>
-      </c>
+      <c r="F1574" t="inlineStr"/>
       <c r="G1574" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -52398,9 +52300,7 @@
       <c r="E1575" t="n">
         <v>2023</v>
       </c>
-      <c r="F1575" t="n">
-        <v>57.1435211987779</v>
-      </c>
+      <c r="F1575" t="inlineStr"/>
       <c r="G1575" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -52431,9 +52331,7 @@
       <c r="E1576" t="n">
         <v>2024</v>
       </c>
-      <c r="F1576" t="n">
-        <v>57.1435211987779</v>
-      </c>
+      <c r="F1576" t="inlineStr"/>
       <c r="G1576" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -53586,9 +53484,7 @@
       <c r="E1611" t="n">
         <v>2024</v>
       </c>
-      <c r="F1611" t="n">
-        <v>22.234</v>
-      </c>
+      <c r="F1611" t="inlineStr"/>
       <c r="G1611" t="inlineStr">
         <is>
           <t>Female Labor Force Participation Rate</t>
@@ -53619,9 +53515,7 @@
       <c r="E1612" t="n">
         <v>1990</v>
       </c>
-      <c r="F1612" t="n">
-        <v>10.553</v>
-      </c>
+      <c r="F1612" t="inlineStr"/>
       <c r="G1612" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -54741,9 +54635,7 @@
       <c r="E1646" t="n">
         <v>2024</v>
       </c>
-      <c r="F1646" t="n">
-        <v>14.48</v>
-      </c>
+      <c r="F1646" t="inlineStr"/>
       <c r="G1646" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -60549,9 +60441,7 @@
       <c r="E1822" t="n">
         <v>1990</v>
       </c>
-      <c r="F1822" t="n">
-        <v>12.96</v>
-      </c>
+      <c r="F1822" t="inlineStr"/>
       <c r="G1822" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -66291,9 +66181,7 @@
       <c r="E1996" t="n">
         <v>2024</v>
       </c>
-      <c r="F1996" t="n">
-        <v>49.398738861084</v>
-      </c>
+      <c r="F1996" t="inlineStr"/>
       <c r="G1996" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -67479,9 +67367,7 @@
       <c r="E2032" t="n">
         <v>1990</v>
       </c>
-      <c r="F2032" t="n">
-        <v>17.374</v>
-      </c>
+      <c r="F2032" t="inlineStr"/>
       <c r="G2032" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>
@@ -73221,9 +73107,7 @@
       <c r="E2206" t="n">
         <v>2024</v>
       </c>
-      <c r="F2206" t="n">
-        <v>109.999862670898</v>
-      </c>
+      <c r="F2206" t="inlineStr"/>
       <c r="G2206" t="inlineStr">
         <is>
           <t>Girls’ Tertiary Enrollment</t>
@@ -74409,9 +74293,7 @@
       <c r="E2242" t="n">
         <v>1990</v>
       </c>
-      <c r="F2242" t="n">
-        <v>7.122</v>
-      </c>
+      <c r="F2242" t="inlineStr"/>
       <c r="G2242" t="inlineStr">
         <is>
           <t>Female Unemployment Rate</t>

</xml_diff>